<commit_message>
Amélioration :reorganisation du dossier afin d'avoir la bd excel à jour sur github pour Christine
</commit_message>
<xml_diff>
--- a/liste_test.xlsx
+++ b/liste_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Etu\Desktop\STAGE_L3_MIASHS_JUSTECHANGE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C069B5-4E66-4EDF-B462-40257AD04CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4FB61C-F889-41E2-846B-083AA96B9C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E8D39404-00AB-45A2-A25F-E5DBF77DE3FC}"/>
+    <workbookView xWindow="5424" yWindow="2412" windowWidth="17280" windowHeight="8880" xr2:uid="{E8D39404-00AB-45A2-A25F-E5DBF77DE3FC}"/>
   </bookViews>
   <sheets>
     <sheet name="tab1_test" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="72">
   <si>
     <t>Ville</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Yasmine TOURNADRE</t>
   </si>
   <si>
-    <t>L'aMie bio</t>
-  </si>
-  <si>
     <t>lamiebionarbonne@hotmail.com</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
     <t>Tel port</t>
   </si>
   <si>
-    <t>Categorie</t>
-  </si>
-  <si>
     <t>Etablissement</t>
   </si>
   <si>
@@ -123,9 +117,6 @@
     <t>Boulangerie</t>
   </si>
   <si>
-    <t>L'Ostal Occitan</t>
-  </si>
-  <si>
     <t>06 45 77 16 15</t>
   </si>
   <si>
@@ -150,9 +141,6 @@
     <t>04 68 65 86 26</t>
   </si>
   <si>
-    <t>Domaine de Craboulette, Route de Marcorignan</t>
-  </si>
-  <si>
     <t>alain@lesabeilles.com</t>
   </si>
   <si>
@@ -165,9 +153,6 @@
     <t>Pourquoi Le CERS</t>
   </si>
   <si>
-    <t>Comptoir</t>
-  </si>
-  <si>
     <t>Non</t>
   </si>
   <si>
@@ -201,9 +186,6 @@
     <t>https://www.facebook.com/boulangerielamiebio/</t>
   </si>
   <si>
-    <t>https://mapausebio.eatbu.com</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/larotisseriedanatole/</t>
   </si>
   <si>
@@ -214,6 +196,63 @@
   </si>
   <si>
     <t>http://o.rouge.free.fr/www/lesabeilles/</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Service</t>
+  </si>
+  <si>
+    <t>Bar</t>
+  </si>
+  <si>
+    <t>Marché</t>
+  </si>
+  <si>
+    <t>Comptoir d'Echange</t>
+  </si>
+  <si>
+    <t>Bien-Etre</t>
+  </si>
+  <si>
+    <t>Sylvain Cara</t>
+  </si>
+  <si>
+    <t>KUPIRIJO parfums</t>
+  </si>
+  <si>
+    <t>06 09 99 10 33</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/parfum_kupirijo/</t>
+  </si>
+  <si>
+    <t>sylvain@kupirijo.com</t>
+  </si>
+  <si>
+    <t>Rue de l'Ancien Courrier</t>
+  </si>
+  <si>
+    <t>La Mie bio</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/mapausebio</t>
+  </si>
+  <si>
+    <t>Contribuer à la vie du quartier</t>
+  </si>
+  <si>
+    <t>Favoriser le commerce local</t>
+  </si>
+  <si>
+    <t>Domaine de Craboules</t>
+  </si>
+  <si>
+    <t>Ostal Occitan</t>
+  </si>
+  <si>
+    <t>Parfumerie</t>
   </si>
 </sst>
 </file>
@@ -474,7 +513,7 @@
     <cellStyle name="Result" xfId="17" xr:uid="{A1687342-5302-464A-8C82-C3A7BA52DD7D}"/>
     <cellStyle name="Result2" xfId="18" xr:uid="{60310D12-4890-4F95-AFD6-0054D16A45A3}"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="17">
     <dxf>
       <font>
         <b val="0"/>
@@ -704,6 +743,78 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <sz val="10"/>
         <color auto="1"/>
         <name val="Arial"/>
@@ -736,13 +847,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71086B8A-17E7-4B80-BBE9-B0590D28D694}" name="Tableau1" displayName="Tableau1" ref="A1:L8" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" headerRowCellStyle="Normal 7" dataCellStyle="Normal 7">
-  <autoFilter ref="A1:L8" xr:uid="{71086B8A-17E7-4B80-BBE9-B0590D28D694}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{128328A1-A6A3-4E31-A665-A3D607B0074B}" name="Responsable" dataDxfId="10" dataCellStyle="Normal 7"/>
-    <tableColumn id="2" xr3:uid="{2C77BE59-DE54-455C-AB09-C65399160FBF}" name="Etablissement" dataDxfId="9" dataCellStyle="Normal 7"/>
-    <tableColumn id="13" xr3:uid="{76CABDBE-30E8-41CA-9C9A-7BDA188BC20D}" name="Comptoir"/>
-    <tableColumn id="11" xr3:uid="{1A18EAFC-90BA-41F7-87D9-7563DBAD802E}" name="Categorie" dataDxfId="8" dataCellStyle="Normal 7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71086B8A-17E7-4B80-BBE9-B0590D28D694}" name="Tableau1" displayName="Tableau1" ref="A1:P9" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normal 7" dataCellStyle="Normal 7">
+  <autoFilter ref="A1:P9" xr:uid="{71086B8A-17E7-4B80-BBE9-B0590D28D694}"/>
+  <tableColumns count="16">
+    <tableColumn id="1" xr3:uid="{128328A1-A6A3-4E31-A665-A3D607B0074B}" name="Responsable" dataDxfId="14" dataCellStyle="Normal 7"/>
+    <tableColumn id="2" xr3:uid="{2C77BE59-DE54-455C-AB09-C65399160FBF}" name="Etablissement" dataDxfId="13" dataCellStyle="Normal 7"/>
+    <tableColumn id="13" xr3:uid="{76CABDBE-30E8-41CA-9C9A-7BDA188BC20D}" name="Centre Culturel"/>
+    <tableColumn id="12" xr3:uid="{18217EAC-34E1-4EBD-B045-C1FE93B2FB29}" name="Alimentation" dataDxfId="12" dataCellStyle="Normal 7"/>
+    <tableColumn id="14" xr3:uid="{15E7D3DE-E7A5-4F86-8A09-0EEF73B788B9}" name="Service" dataDxfId="11" dataCellStyle="Normal 7"/>
+    <tableColumn id="16" xr3:uid="{6454FE71-F76B-43FA-B098-61C9CBC1CCB9}" name="Bien-Etre" dataDxfId="10" dataCellStyle="Normal 7"/>
+    <tableColumn id="15" xr3:uid="{66272DE6-095D-4FEC-92BA-6E860D54537F}" name="Comptoir d'Echange" dataDxfId="9" dataCellStyle="Normal 7"/>
+    <tableColumn id="11" xr3:uid="{1A18EAFC-90BA-41F7-87D9-7563DBAD802E}" name="Description" dataDxfId="8" dataCellStyle="Normal 7"/>
     <tableColumn id="3" xr3:uid="{1CECF1C3-80FE-4939-AB01-745593018426}" name="Tel port" dataDxfId="7" dataCellStyle="Normal 7"/>
     <tableColumn id="4" xr3:uid="{335CF749-49D0-4FEC-9001-F9BBD112CB5C}" name="Liens" dataDxfId="6" dataCellStyle="Normal 7"/>
     <tableColumn id="5" xr3:uid="{825A6221-466B-48FB-BD7B-C5D77916127F}" name="Mail" dataDxfId="5" dataCellStyle="Lien hypertexte"/>
@@ -1053,330 +1168,469 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EB60840-FAE7-4CF5-9026-3D18D3260591}">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="27.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.109375" customWidth="1"/>
-    <col min="4" max="4" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" style="16" customWidth="1"/>
-    <col min="6" max="6" width="40.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="48.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="45" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="33.109375" customWidth="1"/>
+    <col min="8" max="8" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" style="16" customWidth="1"/>
+    <col min="10" max="10" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.44140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="48.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.6">
+    <row r="1" spans="1:16" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="13" t="s">
-        <v>41</v>
+      <c r="P1" s="13" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.6">
+    <row r="2" spans="1:16" ht="15.6">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="18">
+        <v>11100</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="N2" s="24">
+        <v>12</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15.6">
+      <c r="A3" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="J3" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="19">
+        <v>11100</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N3" s="25">
+        <v>3</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" s="9"/>
+    </row>
+    <row r="4" spans="1:16" ht="15.6">
+      <c r="A4" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" s="8">
+        <v>468904312</v>
+      </c>
+      <c r="J4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="18">
+      <c r="L4" s="19">
         <v>11100</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="M4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="24">
-        <v>12</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" s="9"/>
+      <c r="N4" s="25">
+        <v>73</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="P4" s="9"/>
     </row>
-    <row r="3" spans="1:12" ht="15.6">
-      <c r="A3" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="19">
-        <v>11100</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J3" s="25">
-        <v>3</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" s="9"/>
-    </row>
-    <row r="4" spans="1:12" ht="15.6">
-      <c r="A4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="8">
-        <v>468904312</v>
-      </c>
-      <c r="F4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" s="19">
-        <v>11100</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J4" s="25">
-        <v>73</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="L4" s="9"/>
-    </row>
-    <row r="5" spans="1:12" ht="15.6">
+    <row r="5" spans="1:16" ht="15.6">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="5">
+        <v>39</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="5">
         <v>987112083</v>
       </c>
-      <c r="F5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" s="6" t="s">
+      <c r="J5" t="s">
+        <v>66</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="18">
+      <c r="L5" s="18">
         <v>11100</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="M5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="J5" s="24">
+      <c r="N5" s="24">
         <v>41</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="O5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L5" s="9"/>
+      <c r="P5" s="9" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="6" spans="1:12" ht="15.6">
+    <row r="6" spans="1:16" ht="15.6">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5">
+        <v>632354746</v>
+      </c>
+      <c r="J6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="L6" s="18">
+        <v>11100</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="N6" s="24">
+        <v>20</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="15.6">
+      <c r="A7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="20">
+        <v>11100</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="N7" s="26"/>
+      <c r="O7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="15.6">
+      <c r="A8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="L8" s="20">
+        <v>11100</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="N8" s="26">
+        <v>37</v>
+      </c>
+      <c r="O8" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P8" s="9"/>
+    </row>
+    <row r="9" spans="1:16" s="11" customFormat="1" ht="15.6">
+      <c r="A9" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L9" s="21">
+        <v>11100</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="N9" s="27">
+        <v>31</v>
+      </c>
+      <c r="O9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="5">
-        <v>632354746</v>
-      </c>
-      <c r="F6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="18">
-        <v>11100</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="J6" s="24">
-        <v>20</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="15.6">
-      <c r="A7" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="20">
-        <v>11100</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J7" s="26"/>
-      <c r="K7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" s="11" customFormat="1" ht="15.6">
-      <c r="A8" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="21">
-        <v>11100</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="J8" s="27">
-        <v>31</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="L8" s="9"/>
+      <c r="P9" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="12" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{584F290E-4B66-469F-A548-B779B2AB8B16}"/>
-    <hyperlink ref="G6" r:id="rId2" xr:uid="{E7E611C2-3FB6-4C43-8637-1DCEC9F58A9E}"/>
-    <hyperlink ref="G2" r:id="rId3" xr:uid="{4A37D00C-8F85-49F6-A2BD-111396DF0610}"/>
-    <hyperlink ref="G8" r:id="rId4" xr:uid="{CFFD2B09-7097-460D-9E83-065BA665CB8F}"/>
-    <hyperlink ref="G7" r:id="rId5" xr:uid="{741C7A4D-33A0-4B34-A698-7E8EBB796049}"/>
-    <hyperlink ref="G5" r:id="rId6" xr:uid="{9BADF198-2F69-48C6-ADC6-FA84EEBF0A07}"/>
-    <hyperlink ref="G3" r:id="rId7" xr:uid="{C4EAB587-5C48-4256-A119-EA561E4E7A1E}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>